<commit_message>
Improve OCR accuracy with fuzzy number recovery, name-based resolution, and batch-ready pipeline
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20377"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2913FF58-9645-4A47-85D4-B601E0EDD172}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B031593-0C54-4C1F-80B8-FBA0F06DF606}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
   <si>
-    <t>Name</t>
-  </si>
-  <si>
     <t>Department</t>
   </si>
   <si>
@@ -47,6 +44,9 @@
   </si>
   <si>
     <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>EmployeeName</t>
   </si>
 </sst>
 </file>
@@ -374,13 +374,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -388,10 +388,10 @@
         <v>101338</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -399,10 +399,10 @@
         <v>101649</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -410,10 +410,10 @@
         <v>929969</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -421,10 +421,10 @@
         <v>100498</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -432,10 +432,10 @@
         <v>101684</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix OCR anchors and row cropping alignment
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B031593-0C54-4C1F-80B8-FBA0F06DF606}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECEB3C2A-A565-4385-8ACA-B9393211359B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="87">
   <si>
     <t>Department</t>
   </si>
@@ -28,25 +28,259 @@
     <t>CASTHOUSE</t>
   </si>
   <si>
-    <t>Zahid Sarwar</t>
-  </si>
-  <si>
-    <t>Reynaldo Malazarte</t>
-  </si>
-  <si>
-    <t>Wajd AL MAQBALI</t>
-  </si>
-  <si>
-    <t>Abdullah Al Salhi</t>
-  </si>
-  <si>
-    <t>Svetislav Zerzenka</t>
-  </si>
-  <si>
     <t>EmployeeID</t>
   </si>
   <si>
     <t>EmployeeName</t>
+  </si>
+  <si>
+    <t>Ishaq Mohammed</t>
+  </si>
+  <si>
+    <t>Mohammed Al Washahi</t>
+  </si>
+  <si>
+    <t>Mohammed Al Maamari</t>
+  </si>
+  <si>
+    <t>Ali Al Alawi</t>
+  </si>
+  <si>
+    <t>Abdullah Al Reesi</t>
+  </si>
+  <si>
+    <t>Ahmed Al Badi</t>
+  </si>
+  <si>
+    <t>Abdullah AL Harthy</t>
+  </si>
+  <si>
+    <t>Mazyad Al Khan</t>
+  </si>
+  <si>
+    <t>Abdullah Al Maamari</t>
+  </si>
+  <si>
+    <t>Fahad Al Jabri</t>
+  </si>
+  <si>
+    <t>Adil Al Abri</t>
+  </si>
+  <si>
+    <t>Bhaveshkumar Sheth</t>
+  </si>
+  <si>
+    <t>Nabhan Al Jahwari</t>
+  </si>
+  <si>
+    <t>Abdulkareem Al Balushi</t>
+  </si>
+  <si>
+    <t>Mohammed Al Dhahri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABDULLAH AL KALBANI </t>
+  </si>
+  <si>
+    <t>Faiz Al Balushi</t>
+  </si>
+  <si>
+    <t>Ahmed Al Shibli</t>
+  </si>
+  <si>
+    <t>Khalid Al Balushi</t>
+  </si>
+  <si>
+    <t>Bader Al Balushi</t>
+  </si>
+  <si>
+    <t>Ismail Al Balushi</t>
+  </si>
+  <si>
+    <t>Juma Al Abri</t>
+  </si>
+  <si>
+    <t>Sumaiya Al Kindi</t>
+  </si>
+  <si>
+    <t>Patitapaban Samal</t>
+  </si>
+  <si>
+    <t>Khalfan Al Kindi</t>
+  </si>
+  <si>
+    <t>Salim Al Kindi</t>
+  </si>
+  <si>
+    <t>Salim Al Maqbali</t>
+  </si>
+  <si>
+    <t>Said Al Kishri</t>
+  </si>
+  <si>
+    <t>Abdulaziz Al Shamsi</t>
+  </si>
+  <si>
+    <t>Khalid Al Hamdi</t>
+  </si>
+  <si>
+    <t>Hamood Al Maamari</t>
+  </si>
+  <si>
+    <t>Hatim Al Rushdi</t>
+  </si>
+  <si>
+    <t>Hussein Al Balushi</t>
+  </si>
+  <si>
+    <t>Hilal Al Shidi</t>
+  </si>
+  <si>
+    <t>Ali Al Hinai</t>
+  </si>
+  <si>
+    <t>Bilal Al Balushi</t>
+  </si>
+  <si>
+    <t>Maktoom Al Zeidi</t>
+  </si>
+  <si>
+    <t>Nasser Al Maamari</t>
+  </si>
+  <si>
+    <t>Ammar Al Jabri</t>
+  </si>
+  <si>
+    <t>Amur AL Maqbali</t>
+  </si>
+  <si>
+    <t>Nader Al Balushi</t>
+  </si>
+  <si>
+    <t>Jasim Al Marzooqi</t>
+  </si>
+  <si>
+    <t>Darwish Al Maamari</t>
+  </si>
+  <si>
+    <t>Abdullah Al Sharqi</t>
+  </si>
+  <si>
+    <t>Said Al Issai</t>
+  </si>
+  <si>
+    <t>Rashid Al Balushi</t>
+  </si>
+  <si>
+    <t>Veeramalai Dharmalingam</t>
+  </si>
+  <si>
+    <t>Rashid Al Maqbali</t>
+  </si>
+  <si>
+    <t>Abdulaziz Al Balushi</t>
+  </si>
+  <si>
+    <t>Yasir Al Farsi</t>
+  </si>
+  <si>
+    <t>Salim Al Balushi</t>
+  </si>
+  <si>
+    <t>Asaad Al Shidi</t>
+  </si>
+  <si>
+    <t>Mohammed Al Mezaini</t>
+  </si>
+  <si>
+    <t>Yahya Al Saidi</t>
+  </si>
+  <si>
+    <t>Ahmed Al Fezari</t>
+  </si>
+  <si>
+    <t>Ali Al Hosni</t>
+  </si>
+  <si>
+    <t>Balakrishnan Kaliyaperumal</t>
+  </si>
+  <si>
+    <t>Mohammed Navalur</t>
+  </si>
+  <si>
+    <t>Santosh Nalawade</t>
+  </si>
+  <si>
+    <t>Qais Al Khuzaimi</t>
+  </si>
+  <si>
+    <t>Manish Vyas</t>
+  </si>
+  <si>
+    <t>Salim Al Mamari</t>
+  </si>
+  <si>
+    <t>Ahmed Al Dhahri</t>
+  </si>
+  <si>
+    <t>Mustafa Al Farsi</t>
+  </si>
+  <si>
+    <t>Ali Hussain</t>
+  </si>
+  <si>
+    <t>Mohammed Al Risi</t>
+  </si>
+  <si>
+    <t>Hussain AL Shamsi</t>
+  </si>
+  <si>
+    <t>Ahmed AL Shahi</t>
+  </si>
+  <si>
+    <t>Haitham Al Shibly</t>
+  </si>
+  <si>
+    <t>Hamed Al Maamari</t>
+  </si>
+  <si>
+    <t>Shabib Al Maqbali</t>
+  </si>
+  <si>
+    <t>Hamdan Al Badi</t>
+  </si>
+  <si>
+    <t>Mohammed AL Kharusi</t>
+  </si>
+  <si>
+    <t>Mohammed AL Badi</t>
+  </si>
+  <si>
+    <t>Raid AL Farsi</t>
+  </si>
+  <si>
+    <t>Abdullah AL Mamari</t>
+  </si>
+  <si>
+    <t>Khalil AL Balushi</t>
+  </si>
+  <si>
+    <t>Salim AL jabri</t>
+  </si>
+  <si>
+    <t>Khalid Al Sinani</t>
+  </si>
+  <si>
+    <t>Ibrahim Al Balushi</t>
+  </si>
+  <si>
+    <t>Ahmed AL Kaabi</t>
+  </si>
+  <si>
+    <t>Gayth AL Saadi</t>
+  </si>
+  <si>
+    <t>Abdullah Alshibli</t>
   </si>
 </sst>
 </file>
@@ -364,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
@@ -374,10 +608,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -385,10 +619,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>101338</v>
+        <v>100278</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -396,10 +630,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>101649</v>
+        <v>100299</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -407,10 +641,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>929969</v>
+        <v>100416</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>1</v>
@@ -418,10 +652,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>100498</v>
+        <v>100421</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
         <v>1</v>
@@ -429,12 +663,903 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>101684</v>
+        <v>100430</v>
       </c>
       <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>100434</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>100435</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>100438</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>100443</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>100449</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>100457</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>100488</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>100568</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>100626</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>100668</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>100740</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>100742</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>100757</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>100763</v>
+      </c>
+      <c r="B20" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C20" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>100770</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>100771</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>100772</v>
+      </c>
+      <c r="B23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>100774</v>
+      </c>
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>100776</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>100805</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>100818</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>100828</v>
+      </c>
+      <c r="B28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>100842</v>
+      </c>
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>100843</v>
+      </c>
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>100844</v>
+      </c>
+      <c r="B31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>100845</v>
+      </c>
+      <c r="B32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>100847</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>100851</v>
+      </c>
+      <c r="B34" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>100852</v>
+      </c>
+      <c r="B35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>100853</v>
+      </c>
+      <c r="B36" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>100857</v>
+      </c>
+      <c r="B37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>100879</v>
+      </c>
+      <c r="B38" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>100915</v>
+      </c>
+      <c r="B39" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>100937</v>
+      </c>
+      <c r="B40" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>100938</v>
+      </c>
+      <c r="B41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>100943</v>
+      </c>
+      <c r="B42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>100944</v>
+      </c>
+      <c r="B43" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>100945</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>100946</v>
+      </c>
+      <c r="B45" t="s">
+        <v>44</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>100947</v>
+      </c>
+      <c r="B46" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>100948</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>100949</v>
+      </c>
+      <c r="B48" t="s">
+        <v>47</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>100950</v>
+      </c>
+      <c r="B49" t="s">
+        <v>48</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>100954</v>
+      </c>
+      <c r="B50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>100978</v>
+      </c>
+      <c r="B51" t="s">
+        <v>50</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>100980</v>
+      </c>
+      <c r="B52" t="s">
+        <v>51</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>100985</v>
+      </c>
+      <c r="B53" t="s">
+        <v>52</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>101010</v>
+      </c>
+      <c r="B54" t="s">
+        <v>53</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>101011</v>
+      </c>
+      <c r="B55" t="s">
+        <v>54</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>101020</v>
+      </c>
+      <c r="B56" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>101027</v>
+      </c>
+      <c r="B57" t="s">
+        <v>56</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>101043</v>
+      </c>
+      <c r="B58" t="s">
+        <v>57</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>101061</v>
+      </c>
+      <c r="B59" t="s">
+        <v>58</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>101065</v>
+      </c>
+      <c r="B60" t="s">
+        <v>59</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>101098</v>
+      </c>
+      <c r="B61" t="s">
+        <v>60</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>101168</v>
+      </c>
+      <c r="B62" t="s">
+        <v>61</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>101169</v>
+      </c>
+      <c r="B63" t="s">
+        <v>62</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>101213</v>
+      </c>
+      <c r="B64" t="s">
+        <v>63</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>101292</v>
+      </c>
+      <c r="B65" t="s">
+        <v>64</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>101294</v>
+      </c>
+      <c r="B66" t="s">
+        <v>65</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>101306</v>
+      </c>
+      <c r="B67" t="s">
+        <v>66</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>101336</v>
+      </c>
+      <c r="B68" t="s">
+        <v>67</v>
+      </c>
+      <c r="C68" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>101343</v>
+      </c>
+      <c r="B69" t="s">
+        <v>68</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>101388</v>
+      </c>
+      <c r="B70" t="s">
+        <v>69</v>
+      </c>
+      <c r="C70" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>101405</v>
+      </c>
+      <c r="B71" t="s">
+        <v>70</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>101407</v>
+      </c>
+      <c r="B72" t="s">
+        <v>71</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>101483</v>
+      </c>
+      <c r="B73" t="s">
+        <v>72</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>101484</v>
+      </c>
+      <c r="B74" t="s">
+        <v>73</v>
+      </c>
+      <c r="C74" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>101485</v>
+      </c>
+      <c r="B75" t="s">
+        <v>74</v>
+      </c>
+      <c r="C75" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>101487</v>
+      </c>
+      <c r="B76" t="s">
+        <v>75</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>101496</v>
+      </c>
+      <c r="B77" t="s">
+        <v>76</v>
+      </c>
+      <c r="C77" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>101497</v>
+      </c>
+      <c r="B78" t="s">
+        <v>77</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>101533</v>
+      </c>
+      <c r="B79" t="s">
+        <v>78</v>
+      </c>
+      <c r="C79" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>101547</v>
+      </c>
+      <c r="B80" t="s">
+        <v>79</v>
+      </c>
+      <c r="C80" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>101549</v>
+      </c>
+      <c r="B81" t="s">
+        <v>80</v>
+      </c>
+      <c r="C81" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>101553</v>
+      </c>
+      <c r="B82" t="s">
+        <v>81</v>
+      </c>
+      <c r="C82" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>101569</v>
+      </c>
+      <c r="B83" t="s">
+        <v>82</v>
+      </c>
+      <c r="C83" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>101711</v>
+      </c>
+      <c r="B84" t="s">
+        <v>83</v>
+      </c>
+      <c r="C84" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>101715</v>
+      </c>
+      <c r="B85" t="s">
+        <v>84</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>101754</v>
+      </c>
+      <c r="B86" t="s">
+        <v>85</v>
+      </c>
+      <c r="C86" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>101803</v>
+      </c>
+      <c r="B87" t="s">
+        <v>86</v>
+      </c>
+      <c r="C87" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>